<commit_message>
Check agreement between human annotation and split train/val dataset
</commit_message>
<xml_diff>
--- a/scoring/pool_a_177_images.xlsx
+++ b/scoring/pool_a_177_images.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/XiaoJun/avm/scoring/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07D234D1-8F08-FA4B-B2F0-3F50E173DDFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF489C96-EFF5-D647-8809-6A7D16B7F587}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="18360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2267,17 +2267,17 @@
     <col min="4" max="4" width="8" customWidth="1"/>
     <col min="5" max="5" width="22" customWidth="1"/>
     <col min="6" max="6" width="10" customWidth="1"/>
-    <col min="7" max="7" width="14" customWidth="1"/>
-    <col min="8" max="8" width="13" customWidth="1"/>
-    <col min="9" max="9" width="14" customWidth="1"/>
-    <col min="10" max="10" width="13" customWidth="1"/>
-    <col min="11" max="11" width="10" customWidth="1"/>
-    <col min="12" max="12" width="13" customWidth="1"/>
-    <col min="13" max="13" width="45" customWidth="1"/>
-    <col min="14" max="14" width="14" customWidth="1"/>
-    <col min="15" max="15" width="13" customWidth="1"/>
-    <col min="16" max="16" width="14" customWidth="1"/>
-    <col min="17" max="17" width="13" customWidth="1"/>
+    <col min="7" max="7" width="14" hidden="1" customWidth="1"/>
+    <col min="8" max="8" width="13" hidden="1" customWidth="1"/>
+    <col min="9" max="9" width="14" hidden="1" customWidth="1"/>
+    <col min="10" max="10" width="13" hidden="1" customWidth="1"/>
+    <col min="11" max="11" width="10" hidden="1" customWidth="1"/>
+    <col min="12" max="12" width="13" hidden="1" customWidth="1"/>
+    <col min="13" max="13" width="45" hidden="1" customWidth="1"/>
+    <col min="14" max="14" width="14" hidden="1" customWidth="1"/>
+    <col min="15" max="15" width="13" hidden="1" customWidth="1"/>
+    <col min="16" max="16" width="14" hidden="1" customWidth="1"/>
+    <col min="17" max="17" width="13" hidden="1" customWidth="1"/>
     <col min="18" max="18" width="10" customWidth="1"/>
     <col min="19" max="19" width="25" hidden="1" customWidth="1"/>
   </cols>
@@ -2386,7 +2386,7 @@
       <c r="P2" s="6"/>
       <c r="Q2" s="6"/>
       <c r="R2" s="6">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="S2" s="7"/>
     </row>
@@ -2484,7 +2484,7 @@
       <c r="P4" s="6"/>
       <c r="Q4" s="6"/>
       <c r="R4" s="6">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="S4" s="7"/>
     </row>
@@ -2533,7 +2533,7 @@
       <c r="P5" s="6"/>
       <c r="Q5" s="6"/>
       <c r="R5" s="6">
-        <v>7</v>
+        <v>7.5</v>
       </c>
       <c r="S5" s="7"/>
     </row>
@@ -2582,7 +2582,7 @@
       <c r="P6" s="6"/>
       <c r="Q6" s="6"/>
       <c r="R6" s="6">
-        <v>8</v>
+        <v>8.5</v>
       </c>
       <c r="S6" s="7"/>
     </row>
@@ -2778,7 +2778,7 @@
       <c r="P10" s="6"/>
       <c r="Q10" s="6"/>
       <c r="R10" s="6">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="S10" s="7"/>
     </row>
@@ -2827,7 +2827,7 @@
       <c r="P11" s="6"/>
       <c r="Q11" s="6"/>
       <c r="R11" s="6">
-        <v>7.5</v>
+        <v>8</v>
       </c>
       <c r="S11" s="7"/>
     </row>
@@ -2876,7 +2876,7 @@
       <c r="P12" s="6"/>
       <c r="Q12" s="6"/>
       <c r="R12" s="6">
-        <v>7.5</v>
+        <v>8</v>
       </c>
       <c r="S12" s="7"/>
     </row>
@@ -2925,7 +2925,7 @@
       <c r="P13" s="6"/>
       <c r="Q13" s="6"/>
       <c r="R13" s="6">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="S13" s="7"/>
     </row>
@@ -2974,7 +2974,7 @@
       <c r="P14" s="6"/>
       <c r="Q14" s="6"/>
       <c r="R14" s="6">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="S14" s="7"/>
     </row>
@@ -3023,7 +3023,7 @@
       <c r="P15" s="6"/>
       <c r="Q15" s="6"/>
       <c r="R15" s="6">
-        <v>7</v>
+        <v>7.5</v>
       </c>
       <c r="S15" s="7"/>
     </row>
@@ -3219,7 +3219,7 @@
       <c r="P19" s="6"/>
       <c r="Q19" s="6"/>
       <c r="R19" s="6">
-        <v>7.5</v>
+        <v>8</v>
       </c>
       <c r="S19" s="7"/>
     </row>
@@ -3268,7 +3268,7 @@
       <c r="P20" s="6"/>
       <c r="Q20" s="6"/>
       <c r="R20" s="6">
-        <v>7</v>
+        <v>7.5</v>
       </c>
       <c r="S20" s="7"/>
     </row>
@@ -3415,7 +3415,7 @@
       <c r="P23" s="6"/>
       <c r="Q23" s="6"/>
       <c r="R23" s="6">
-        <v>9.5</v>
+        <v>8</v>
       </c>
       <c r="S23" s="7"/>
     </row>
@@ -3464,7 +3464,7 @@
       <c r="P24" s="6"/>
       <c r="Q24" s="6"/>
       <c r="R24" s="6">
-        <v>7</v>
+        <v>7.5</v>
       </c>
       <c r="S24" s="7"/>
     </row>
@@ -3513,7 +3513,7 @@
       <c r="P25" s="6"/>
       <c r="Q25" s="6"/>
       <c r="R25" s="6">
-        <v>6.5</v>
+        <v>6</v>
       </c>
       <c r="S25" s="7"/>
     </row>
@@ -3611,7 +3611,7 @@
       <c r="P27" s="6"/>
       <c r="Q27" s="6"/>
       <c r="R27" s="6">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="S27" s="7"/>
     </row>
@@ -3660,7 +3660,7 @@
       <c r="P28" s="6"/>
       <c r="Q28" s="6"/>
       <c r="R28" s="6">
-        <v>7.5</v>
+        <v>8.5</v>
       </c>
       <c r="S28" s="7"/>
     </row>
@@ -3709,7 +3709,7 @@
       <c r="P29" s="6"/>
       <c r="Q29" s="6"/>
       <c r="R29" s="6">
-        <v>8</v>
+        <v>8.5</v>
       </c>
       <c r="S29" s="7"/>
     </row>
@@ -3807,7 +3807,7 @@
       <c r="P31" s="6"/>
       <c r="Q31" s="6"/>
       <c r="R31" s="6">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="S31" s="7"/>
     </row>
@@ -3856,7 +3856,7 @@
       <c r="P32" s="6"/>
       <c r="Q32" s="6"/>
       <c r="R32" s="6">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="S32" s="7"/>
     </row>
@@ -3905,7 +3905,7 @@
       <c r="P33" s="6"/>
       <c r="Q33" s="6"/>
       <c r="R33" s="6">
-        <v>8</v>
+        <v>8.5</v>
       </c>
       <c r="S33" s="7"/>
     </row>
@@ -4052,7 +4052,7 @@
       <c r="P36" s="6"/>
       <c r="Q36" s="6"/>
       <c r="R36" s="6">
-        <v>8</v>
+        <v>8.5</v>
       </c>
       <c r="S36" s="7"/>
     </row>
@@ -4101,7 +4101,7 @@
       <c r="P37" s="6"/>
       <c r="Q37" s="6"/>
       <c r="R37" s="6">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="S37" s="7"/>
     </row>
@@ -4150,7 +4150,7 @@
       <c r="P38" s="6"/>
       <c r="Q38" s="6"/>
       <c r="R38" s="6">
-        <v>7.5</v>
+        <v>8</v>
       </c>
       <c r="S38" s="7"/>
     </row>
@@ -4199,7 +4199,7 @@
       <c r="P39" s="6"/>
       <c r="Q39" s="6"/>
       <c r="R39" s="6">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="S39" s="7"/>
     </row>
@@ -4248,7 +4248,7 @@
       <c r="P40" s="6"/>
       <c r="Q40" s="6"/>
       <c r="R40" s="6">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="S40" s="7"/>
     </row>
@@ -4346,7 +4346,7 @@
       <c r="P42" s="6"/>
       <c r="Q42" s="6"/>
       <c r="R42" s="6">
-        <v>8</v>
+        <v>8.5</v>
       </c>
       <c r="S42" s="7"/>
     </row>
@@ -4493,7 +4493,7 @@
       <c r="P45" s="6"/>
       <c r="Q45" s="6"/>
       <c r="R45" s="6">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="S45" s="7"/>
     </row>
@@ -4885,7 +4885,7 @@
       <c r="P53" s="6"/>
       <c r="Q53" s="6"/>
       <c r="R53" s="6">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="S53" s="7"/>
     </row>
@@ -4934,7 +4934,7 @@
       <c r="P54" s="6"/>
       <c r="Q54" s="6"/>
       <c r="R54" s="6">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="S54" s="7"/>
     </row>
@@ -4983,7 +4983,7 @@
       <c r="P55" s="6"/>
       <c r="Q55" s="6"/>
       <c r="R55" s="6">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="S55" s="7"/>
     </row>
@@ -5081,7 +5081,7 @@
       <c r="P57" s="6"/>
       <c r="Q57" s="6"/>
       <c r="R57" s="6">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="S57" s="7"/>
     </row>
@@ -5130,7 +5130,7 @@
       <c r="P58" s="6"/>
       <c r="Q58" s="6"/>
       <c r="R58" s="6">
-        <v>7.5</v>
+        <v>8</v>
       </c>
       <c r="S58" s="7"/>
     </row>
@@ -5179,7 +5179,7 @@
       <c r="P59" s="6"/>
       <c r="Q59" s="6"/>
       <c r="R59" s="6">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="S59" s="7"/>
     </row>
@@ -5228,7 +5228,7 @@
       <c r="P60" s="6"/>
       <c r="Q60" s="6"/>
       <c r="R60" s="6">
-        <v>8</v>
+        <v>8.5</v>
       </c>
       <c r="S60" s="7"/>
     </row>
@@ -5277,7 +5277,7 @@
       <c r="P61" s="6"/>
       <c r="Q61" s="6"/>
       <c r="R61" s="6">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="S61" s="7"/>
     </row>
@@ -5326,7 +5326,7 @@
       <c r="P62" s="6"/>
       <c r="Q62" s="6"/>
       <c r="R62" s="6">
-        <v>8.5</v>
+        <v>8.75</v>
       </c>
       <c r="S62" s="7"/>
     </row>
@@ -5424,7 +5424,7 @@
       <c r="P64" s="6"/>
       <c r="Q64" s="6"/>
       <c r="R64" s="6">
-        <v>7.5</v>
+        <v>8</v>
       </c>
       <c r="S64" s="7"/>
     </row>
@@ -5522,7 +5522,7 @@
       <c r="P66" s="6"/>
       <c r="Q66" s="6"/>
       <c r="R66" s="6">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="S66" s="7"/>
     </row>
@@ -5669,7 +5669,7 @@
       <c r="P69" s="6"/>
       <c r="Q69" s="6"/>
       <c r="R69" s="6">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="S69" s="7"/>
     </row>
@@ -5718,7 +5718,7 @@
       <c r="P70" s="6"/>
       <c r="Q70" s="6"/>
       <c r="R70" s="6">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="S70" s="7"/>
     </row>
@@ -6306,7 +6306,7 @@
       <c r="P82" s="6"/>
       <c r="Q82" s="6"/>
       <c r="R82" s="6">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="S82" s="7"/>
     </row>
@@ -6355,7 +6355,7 @@
       <c r="P83" s="6"/>
       <c r="Q83" s="6"/>
       <c r="R83" s="6">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="S83" s="7"/>
     </row>
@@ -6502,7 +6502,7 @@
       <c r="P86" s="6"/>
       <c r="Q86" s="6"/>
       <c r="R86" s="6">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="S86" s="7"/>
     </row>
@@ -6551,7 +6551,7 @@
       <c r="P87" s="6"/>
       <c r="Q87" s="6"/>
       <c r="R87" s="6">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="S87" s="7"/>
     </row>
@@ -6600,7 +6600,7 @@
       <c r="P88" s="6"/>
       <c r="Q88" s="6"/>
       <c r="R88" s="6">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="S88" s="7"/>
     </row>
@@ -7041,7 +7041,7 @@
       <c r="P97" s="6"/>
       <c r="Q97" s="6"/>
       <c r="R97" s="6">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="S97" s="7"/>
     </row>
@@ -7090,7 +7090,7 @@
       <c r="P98" s="6"/>
       <c r="Q98" s="6"/>
       <c r="R98" s="6">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="S98" s="7"/>
     </row>
@@ -7188,7 +7188,7 @@
       <c r="P100" s="6"/>
       <c r="Q100" s="6"/>
       <c r="R100" s="6">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="S100" s="7"/>
     </row>
@@ -7237,7 +7237,7 @@
       <c r="P101" s="6"/>
       <c r="Q101" s="6"/>
       <c r="R101" s="6">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="S101" s="7"/>
     </row>
@@ -7335,7 +7335,7 @@
       <c r="P103" s="6"/>
       <c r="Q103" s="6"/>
       <c r="R103" s="6">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="S103" s="7"/>
     </row>
@@ -7384,7 +7384,7 @@
       <c r="P104" s="6"/>
       <c r="Q104" s="6"/>
       <c r="R104" s="6">
-        <v>6</v>
+        <v>4.5</v>
       </c>
       <c r="S104" s="7"/>
     </row>
@@ -7433,7 +7433,7 @@
       <c r="P105" s="6"/>
       <c r="Q105" s="6"/>
       <c r="R105" s="6">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="S105" s="7"/>
     </row>
@@ -7482,7 +7482,7 @@
       <c r="P106" s="6"/>
       <c r="Q106" s="6"/>
       <c r="R106" s="6">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="S106" s="7"/>
     </row>
@@ -7531,7 +7531,7 @@
       <c r="P107" s="6"/>
       <c r="Q107" s="6"/>
       <c r="R107" s="6">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="S107" s="7"/>
     </row>
@@ -7580,7 +7580,7 @@
       <c r="P108" s="6"/>
       <c r="Q108" s="6"/>
       <c r="R108" s="6">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="S108" s="7"/>
     </row>
@@ -7629,7 +7629,7 @@
       <c r="P109" s="6"/>
       <c r="Q109" s="6"/>
       <c r="R109" s="6">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="S109" s="7"/>
     </row>
@@ -7678,7 +7678,7 @@
       <c r="P110" s="6"/>
       <c r="Q110" s="6"/>
       <c r="R110" s="6">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="S110" s="7"/>
     </row>
@@ -7727,7 +7727,7 @@
       <c r="P111" s="6"/>
       <c r="Q111" s="6"/>
       <c r="R111" s="6">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="S111" s="7"/>
     </row>
@@ -7825,7 +7825,7 @@
       <c r="P113" s="6"/>
       <c r="Q113" s="6"/>
       <c r="R113" s="6">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="S113" s="7"/>
     </row>
@@ -7923,7 +7923,7 @@
       <c r="P115" s="6"/>
       <c r="Q115" s="6"/>
       <c r="R115" s="6">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="S115" s="7"/>
     </row>
@@ -7972,7 +7972,7 @@
       <c r="P116" s="6"/>
       <c r="Q116" s="6"/>
       <c r="R116" s="6">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="S116" s="7"/>
     </row>
@@ -8021,7 +8021,7 @@
       <c r="P117" s="6"/>
       <c r="Q117" s="6"/>
       <c r="R117" s="6">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="S117" s="7"/>
     </row>
@@ -8070,7 +8070,7 @@
       <c r="P118" s="6"/>
       <c r="Q118" s="6"/>
       <c r="R118" s="6">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="S118" s="7"/>
     </row>
@@ -8119,7 +8119,7 @@
       <c r="P119" s="6"/>
       <c r="Q119" s="6"/>
       <c r="R119" s="6">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="S119" s="7"/>
     </row>
@@ -8168,7 +8168,7 @@
       <c r="P120" s="6"/>
       <c r="Q120" s="6"/>
       <c r="R120" s="6">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="S120" s="7"/>
     </row>
@@ -8217,7 +8217,7 @@
       <c r="P121" s="6"/>
       <c r="Q121" s="6"/>
       <c r="R121" s="6">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="S121" s="7"/>
     </row>
@@ -8266,7 +8266,7 @@
       <c r="P122" s="6"/>
       <c r="Q122" s="6"/>
       <c r="R122" s="6">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S122" s="7"/>
     </row>
@@ -8364,7 +8364,7 @@
       <c r="P124" s="6"/>
       <c r="Q124" s="6"/>
       <c r="R124" s="6">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="S124" s="7"/>
     </row>
@@ -8462,7 +8462,7 @@
       <c r="P126" s="6"/>
       <c r="Q126" s="6"/>
       <c r="R126" s="6">
-        <v>8</v>
+        <v>6.5</v>
       </c>
       <c r="S126" s="7"/>
     </row>
@@ -8511,7 +8511,7 @@
       <c r="P127" s="6"/>
       <c r="Q127" s="6"/>
       <c r="R127" s="6">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="S127" s="7"/>
     </row>
@@ -8707,7 +8707,7 @@
       <c r="P131" s="6"/>
       <c r="Q131" s="6"/>
       <c r="R131" s="6">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="S131" s="7"/>
     </row>
@@ -8756,7 +8756,7 @@
       <c r="P132" s="6"/>
       <c r="Q132" s="6"/>
       <c r="R132" s="6">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S132" s="7"/>
     </row>
@@ -8854,7 +8854,7 @@
       <c r="P134" s="6"/>
       <c r="Q134" s="6"/>
       <c r="R134" s="6">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="S134" s="7"/>
     </row>
@@ -8903,7 +8903,7 @@
       <c r="P135" s="6"/>
       <c r="Q135" s="6"/>
       <c r="R135" s="6">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="S135" s="7"/>
     </row>
@@ -8952,7 +8952,7 @@
       <c r="P136" s="6"/>
       <c r="Q136" s="6"/>
       <c r="R136" s="6">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="S136" s="7"/>
     </row>
@@ -9001,7 +9001,7 @@
       <c r="P137" s="6"/>
       <c r="Q137" s="6"/>
       <c r="R137" s="6">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="S137" s="7"/>
     </row>
@@ -9050,7 +9050,7 @@
       <c r="P138" s="6"/>
       <c r="Q138" s="6"/>
       <c r="R138" s="6">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="S138" s="7"/>
     </row>
@@ -9099,7 +9099,7 @@
       <c r="P139" s="6"/>
       <c r="Q139" s="6"/>
       <c r="R139" s="6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S139" s="7"/>
     </row>
@@ -9148,7 +9148,7 @@
       <c r="P140" s="6"/>
       <c r="Q140" s="6"/>
       <c r="R140" s="6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S140" s="7"/>
     </row>
@@ -9246,7 +9246,7 @@
       <c r="P142" s="6"/>
       <c r="Q142" s="6"/>
       <c r="R142" s="6">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="S142" s="7"/>
     </row>
@@ -9295,7 +9295,7 @@
       <c r="P143" s="6"/>
       <c r="Q143" s="6"/>
       <c r="R143" s="6">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="S143" s="7"/>
     </row>
@@ -9393,7 +9393,7 @@
       <c r="P145" s="6"/>
       <c r="Q145" s="6"/>
       <c r="R145" s="6">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="S145" s="7"/>
     </row>
@@ -9687,7 +9687,7 @@
       <c r="P151" s="6"/>
       <c r="Q151" s="6"/>
       <c r="R151" s="6">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="S151" s="7"/>
     </row>
@@ -9736,7 +9736,7 @@
       <c r="P152" s="6"/>
       <c r="Q152" s="6"/>
       <c r="R152" s="6">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="S152" s="7"/>
     </row>
@@ -9785,7 +9785,7 @@
       <c r="P153" s="6"/>
       <c r="Q153" s="6"/>
       <c r="R153" s="6">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="S153" s="7"/>
     </row>
@@ -9834,7 +9834,7 @@
       <c r="P154" s="6"/>
       <c r="Q154" s="6"/>
       <c r="R154" s="6">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="S154" s="7"/>
     </row>
@@ -10471,7 +10471,7 @@
       <c r="P167" s="6"/>
       <c r="Q167" s="6"/>
       <c r="R167" s="6">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="S167" s="7"/>
     </row>
@@ -10520,7 +10520,7 @@
       <c r="P168" s="6"/>
       <c r="Q168" s="6"/>
       <c r="R168" s="6">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="S168" s="7"/>
     </row>
@@ -10618,7 +10618,7 @@
       <c r="P170" s="6"/>
       <c r="Q170" s="6"/>
       <c r="R170" s="6">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="S170" s="7"/>
     </row>
@@ -10667,7 +10667,7 @@
       <c r="P171" s="6"/>
       <c r="Q171" s="6"/>
       <c r="R171" s="6">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="S171" s="7"/>
     </row>
@@ -10863,7 +10863,7 @@
       <c r="P175" s="6"/>
       <c r="Q175" s="6"/>
       <c r="R175" s="6">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="S175" s="7"/>
     </row>
@@ -10912,7 +10912,7 @@
       <c r="P176" s="6"/>
       <c r="Q176" s="6"/>
       <c r="R176" s="6">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="S176" s="7"/>
     </row>

</xml_diff>